<commit_message>
Add comprehensive analysis pipeline and validation tools for AD Model v3
This update includes:
- Updated manuscript files (Word, Markdown, LaTeX) with latest revisions
- New full analysis pipeline (run_full_analysis.py) for complete model execution
- Figure generation scripts for manuscript Figures 2, 3, and 4
- Age distribution and prevalence validation tools
- ONS projection data integration
- Reorganized PSA results from root to AD_Model_v3 folder
- Cleanup utilities for duplicate PSA files
- Test pipeline for model validation
- Generated validation plots and data exports
- Documentation updates (README, data export guide, LaTeX update summary)

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AD_Study/v3/pd_sensitivity_analysis.xlsx
+++ b/AD_Study/v3/pd_sensitivity_analysis.xlsx
@@ -545,34 +545,34 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>340566785278.2333</v>
+        <v>320861637534.9702</v>
       </c>
       <c r="B2" t="n">
-        <v>268125310463.219</v>
+        <v>245678593291.699</v>
       </c>
       <c r="C2" t="n">
-        <v>141375597.2741284</v>
+        <v>163118311.5350502</v>
       </c>
       <c r="D2" t="n">
-        <v>10196048.12406609</v>
+        <v>9159176.181840597</v>
       </c>
       <c r="E2" t="n">
-        <v>2779782</v>
+        <v>2351610</v>
       </c>
       <c r="F2" t="n">
-        <v>608692095741.4523</v>
+        <v>566540230826.6692</v>
       </c>
       <c r="G2" t="n">
-        <v>151571645.3981945</v>
+        <v>172277487.7168908</v>
       </c>
       <c r="H2" t="n">
-        <v>413881</v>
+        <v>363390</v>
       </c>
       <c r="I2" t="n">
-        <v>492318</v>
+        <v>413072</v>
       </c>
       <c r="J2" t="n">
-        <v>530861</v>
+        <v>490265</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -593,34 +593,34 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>306818718978.9903</v>
+        <v>293225194585.9003</v>
       </c>
       <c r="B3" t="n">
-        <v>244757483903.798</v>
+        <v>227575815487.3014</v>
       </c>
       <c r="C3" t="n">
-        <v>137010344.1794153</v>
+        <v>160326704.9279528</v>
       </c>
       <c r="D3" t="n">
-        <v>9312173.992738904</v>
+        <v>8490437.267896965</v>
       </c>
       <c r="E3" t="n">
-        <v>2544945</v>
+        <v>2183398</v>
       </c>
       <c r="F3" t="n">
-        <v>551576202882.7883</v>
+        <v>520801010073.2018</v>
       </c>
       <c r="G3" t="n">
-        <v>146322518.1721542</v>
+        <v>168817142.1958498</v>
       </c>
       <c r="H3" t="n">
-        <v>371067</v>
+        <v>340276</v>
       </c>
       <c r="I3" t="n">
-        <v>462934</v>
+        <v>394001</v>
       </c>
       <c r="J3" t="n">
-        <v>486342</v>
+        <v>460819</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -641,34 +641,34 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>321584040922.4578</v>
+        <v>307336489736.7234</v>
       </c>
       <c r="B4" t="n">
-        <v>256705678365.0472</v>
+        <v>238830664970.3009</v>
       </c>
       <c r="C4" t="n">
-        <v>136784210.0330866</v>
+        <v>160123552.3687093</v>
       </c>
       <c r="D4" t="n">
-        <v>9799130.69617559</v>
+        <v>8944178.463179268</v>
       </c>
       <c r="E4" t="n">
-        <v>2701735</v>
+        <v>2322813</v>
       </c>
       <c r="F4" t="n">
-        <v>578289719287.5049</v>
+        <v>546167154707.0244</v>
       </c>
       <c r="G4" t="n">
-        <v>146583340.7292622</v>
+        <v>169067730.8318886</v>
       </c>
       <c r="H4" t="n">
-        <v>392588</v>
+        <v>361727</v>
       </c>
       <c r="I4" t="n">
-        <v>486620</v>
+        <v>417133</v>
       </c>
       <c r="J4" t="n">
-        <v>514432</v>
+        <v>487945</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -689,34 +689,34 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>351492424877.7624</v>
+        <v>330472121741.2192</v>
       </c>
       <c r="B5" t="n">
-        <v>276936332316.0852</v>
+        <v>253772042891.3088</v>
       </c>
       <c r="C5" t="n">
-        <v>141219491.3728628</v>
+        <v>162949034.1985876</v>
       </c>
       <c r="D5" t="n">
-        <v>10551499.40202724</v>
+        <v>9481282.741506612</v>
       </c>
       <c r="E5" t="n">
-        <v>2894596</v>
+        <v>2447052</v>
       </c>
       <c r="F5" t="n">
-        <v>628428757193.8477</v>
+        <v>584244164632.528</v>
       </c>
       <c r="G5" t="n">
-        <v>151770990.7748901</v>
+        <v>172430316.9400942</v>
       </c>
       <c r="H5" t="n">
-        <v>428653</v>
+        <v>377506</v>
       </c>
       <c r="I5" t="n">
-        <v>511696</v>
+        <v>428932</v>
       </c>
       <c r="J5" t="n">
-        <v>552002</v>
+        <v>508922</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -737,34 +737,34 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>310402130129.2218</v>
+        <v>296823320241.7306</v>
       </c>
       <c r="B6" t="n">
-        <v>247735772340.671</v>
+        <v>230241625059.67</v>
       </c>
       <c r="C6" t="n">
-        <v>136968559.5589452</v>
+        <v>160295583.2892801</v>
       </c>
       <c r="D6" t="n">
-        <v>9430100.222330146</v>
+        <v>8600057.366235413</v>
       </c>
       <c r="E6" t="n">
-        <v>2582837</v>
+        <v>2218198</v>
       </c>
       <c r="F6" t="n">
-        <v>558137902469.8928</v>
+        <v>527064945301.4006</v>
       </c>
       <c r="G6" t="n">
-        <v>146398659.7812754</v>
+        <v>168895640.6555156</v>
       </c>
       <c r="H6" t="n">
-        <v>375774</v>
+        <v>346689</v>
       </c>
       <c r="I6" t="n">
-        <v>467529</v>
+        <v>399433</v>
       </c>
       <c r="J6" t="n">
-        <v>494144</v>
+        <v>467743</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -785,34 +785,34 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>339806251867.5485</v>
+        <v>325127823796.4399</v>
       </c>
       <c r="B7" t="n">
-        <v>271245280090.3494</v>
+        <v>252263902629.9138</v>
       </c>
       <c r="C7" t="n">
-        <v>136513710.7183905</v>
+        <v>159836295.469596</v>
       </c>
       <c r="D7" t="n">
-        <v>10394266.97009572</v>
+        <v>9483038.439992327</v>
       </c>
       <c r="E7" t="n">
-        <v>2894042</v>
+        <v>2490613</v>
       </c>
       <c r="F7" t="n">
-        <v>611051531957.8979</v>
+        <v>577391726426.3538</v>
       </c>
       <c r="G7" t="n">
-        <v>146907977.6884862</v>
+        <v>169319333.9095883</v>
       </c>
       <c r="H7" t="n">
-        <v>419517</v>
+        <v>386140</v>
       </c>
       <c r="I7" t="n">
-        <v>518612</v>
+        <v>445354</v>
       </c>
       <c r="J7" t="n">
-        <v>548732</v>
+        <v>521818</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -833,34 +833,34 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>362342747194.3394</v>
+        <v>340445541691.2623</v>
       </c>
       <c r="B8" t="n">
-        <v>285703712034.7458</v>
+        <v>261471383359.2565</v>
       </c>
       <c r="C8" t="n">
-        <v>141049337.9619422</v>
+        <v>162785001.648433</v>
       </c>
       <c r="D8" t="n">
-        <v>10904369.06807779</v>
+        <v>9787776.790610945</v>
       </c>
       <c r="E8" t="n">
-        <v>3007517</v>
+        <v>2542248</v>
       </c>
       <c r="F8" t="n">
-        <v>648046459229.0852</v>
+        <v>601916925050.5188</v>
       </c>
       <c r="G8" t="n">
-        <v>151953707.03002</v>
+        <v>172572778.4390439</v>
       </c>
       <c r="H8" t="n">
-        <v>445619</v>
+        <v>392023</v>
       </c>
       <c r="I8" t="n">
-        <v>529205</v>
+        <v>444558</v>
       </c>
       <c r="J8" t="n">
-        <v>572832</v>
+        <v>526086</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -881,34 +881,34 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>314108373312.0554</v>
+        <v>299699841069.0864</v>
       </c>
       <c r="B9" t="n">
-        <v>250459390463.355</v>
+        <v>232929343463.4925</v>
       </c>
       <c r="C9" t="n">
-        <v>136915148.8427759</v>
+        <v>160228927.8513737</v>
       </c>
       <c r="D9" t="n">
-        <v>9545927.863455219</v>
+        <v>8707264.924061259</v>
       </c>
       <c r="E9" t="n">
-        <v>2621631</v>
+        <v>2249704</v>
       </c>
       <c r="F9" t="n">
-        <v>564567763775.4104</v>
+        <v>532629184532.5789</v>
       </c>
       <c r="G9" t="n">
-        <v>146461076.7062311</v>
+        <v>168936192.775435</v>
       </c>
       <c r="H9" t="n">
-        <v>381673</v>
+        <v>350902</v>
       </c>
       <c r="I9" t="n">
-        <v>473726</v>
+        <v>404410</v>
       </c>
       <c r="J9" t="n">
-        <v>500503</v>
+        <v>474461</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -929,34 +929,34 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>358208588975.2632</v>
+        <v>342386119363.3699</v>
       </c>
       <c r="B10" t="n">
-        <v>285750385018.336</v>
+        <v>265514717360.704</v>
       </c>
       <c r="C10" t="n">
-        <v>136230776.0909806</v>
+        <v>159565382.0897255</v>
       </c>
       <c r="D10" t="n">
-        <v>10981842.40099476</v>
+        <v>10015112.93354905</v>
       </c>
       <c r="E10" t="n">
-        <v>3087083</v>
+        <v>2658208</v>
       </c>
       <c r="F10" t="n">
-        <v>643958973993.5991</v>
+        <v>607900836724.074</v>
       </c>
       <c r="G10" t="n">
-        <v>147212618.4919753</v>
+        <v>169580495.0232745</v>
       </c>
       <c r="H10" t="n">
-        <v>446937</v>
+        <v>413823</v>
       </c>
       <c r="I10" t="n">
-        <v>549989</v>
+        <v>472373</v>
       </c>
       <c r="J10" t="n">
-        <v>581390</v>
+        <v>552480</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1187,43 +1187,43 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>340566785278.2333</v>
+        <v>320861637534.9702</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>268125310463.219</v>
+        <v>245678593291.699</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>141375597.2741284</v>
+        <v>163118311.5350502</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>10196048.12406609</v>
+        <v>9159176.181840597</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>2779782</v>
+        <v>2351610</v>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>608692095741.4523</v>
+        <v>566540230826.6692</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
-        <v>151571645.3981945</v>
+        <v>172277487.7168908</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>413881</v>
+        <v>363390</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>492318</v>
+        <v>413072</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>530861</v>
+        <v>490265</v>
       </c>
       <c r="W4" t="inlineStr"/>
     </row>
@@ -1240,43 +1240,43 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>321584040922.4578</v>
+        <v>307336489736.7234</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>256705678365.0472</v>
+        <v>238830664970.3009</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>136784210.0330866</v>
+        <v>160123552.3687093</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>9799130.69617559</v>
+        <v>8944178.463179268</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>2701735</v>
+        <v>2322813</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
-        <v>578289719287.5049</v>
+        <v>546167154707.0244</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
-        <v>146583340.7292622</v>
+        <v>169067730.8318886</v>
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="n">
-        <v>392588</v>
+        <v>361727</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
-        <v>486620</v>
+        <v>417133</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>514432</v>
+        <v>487945</v>
       </c>
       <c r="W5" t="inlineStr"/>
     </row>
@@ -1289,43 +1289,43 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>306818718978.9903</v>
+        <v>293225194585.9003</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>244757483903.798</v>
+        <v>227575815487.3014</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>137010344.1794153</v>
+        <v>160326704.9279528</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>9312173.992738904</v>
+        <v>8490437.267896965</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
-        <v>2544945</v>
+        <v>2183398</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
-        <v>551576202882.7883</v>
+        <v>520801010073.2018</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
-        <v>146322518.1721542</v>
+        <v>168817142.1958498</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="n">
-        <v>371067</v>
+        <v>340276</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
-        <v>462934</v>
+        <v>394001</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>486342</v>
+        <v>460819</v>
       </c>
       <c r="W6" t="inlineStr"/>
     </row>
@@ -1344,43 +1344,43 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>351492424877.7624</v>
+        <v>330472121741.2192</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>276936332316.0852</v>
+        <v>253772042891.3088</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>141219491.3728628</v>
+        <v>162949034.1985876</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="n">
-        <v>10551499.40202724</v>
+        <v>9481282.741506612</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>2894596</v>
+        <v>2447052</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>628428757193.8477</v>
+        <v>584244164632.528</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
-        <v>151770990.7748901</v>
+        <v>172430316.9400942</v>
       </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="n">
-        <v>428653</v>
+        <v>377506</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
-        <v>511696</v>
+        <v>428932</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>552002</v>
+        <v>508922</v>
       </c>
       <c r="W7" t="inlineStr"/>
     </row>
@@ -1397,43 +1397,43 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>339806251867.5485</v>
+        <v>325127823796.4399</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>271245280090.3494</v>
+        <v>252263902629.9138</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>136513710.7183905</v>
+        <v>159836295.469596</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>10394266.97009572</v>
+        <v>9483038.439992327</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>2894042</v>
+        <v>2490613</v>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>611051531957.8979</v>
+        <v>577391726426.3538</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
-        <v>146907977.6884862</v>
+        <v>169319333.9095883</v>
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="n">
-        <v>419517</v>
+        <v>386140</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
-        <v>518612</v>
+        <v>445354</v>
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>548732</v>
+        <v>521818</v>
       </c>
       <c r="W8" t="inlineStr"/>
     </row>
@@ -1446,43 +1446,43 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>310402130129.2218</v>
+        <v>296823320241.7306</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>247735772340.671</v>
+        <v>230241625059.67</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>136968559.5589452</v>
+        <v>160295583.2892801</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="n">
-        <v>9430100.222330146</v>
+        <v>8600057.366235413</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>2582837</v>
+        <v>2218198</v>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
-        <v>558137902469.8928</v>
+        <v>527064945301.4006</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
-        <v>146398659.7812754</v>
+        <v>168895640.6555156</v>
       </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="n">
-        <v>375774</v>
+        <v>346689</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>467529</v>
+        <v>399433</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>494144</v>
+        <v>467743</v>
       </c>
       <c r="W9" t="inlineStr"/>
     </row>
@@ -1501,43 +1501,43 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>362342747194.3394</v>
+        <v>340445541691.2623</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>285703712034.7458</v>
+        <v>261471383359.2565</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>141049337.9619422</v>
+        <v>162785001.648433</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="n">
-        <v>10904369.06807779</v>
+        <v>9787776.790610945</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
-        <v>3007517</v>
+        <v>2542248</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
-        <v>648046459229.0852</v>
+        <v>601916925050.5188</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
-        <v>151953707.03002</v>
+        <v>172572778.4390439</v>
       </c>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="n">
-        <v>445619</v>
+        <v>392023</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
-        <v>529205</v>
+        <v>444558</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>572832</v>
+        <v>526086</v>
       </c>
       <c r="W10" t="inlineStr"/>
     </row>
@@ -1554,43 +1554,43 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>358208588975.2632</v>
+        <v>342386119363.3699</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>285750385018.336</v>
+        <v>265514717360.704</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>136230776.0909806</v>
+        <v>159565382.0897255</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>10981842.40099476</v>
+        <v>10015112.93354905</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>3087083</v>
+        <v>2658208</v>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
-        <v>643958973993.5991</v>
+        <v>607900836724.074</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
-        <v>147212618.4919753</v>
+        <v>169580495.0232745</v>
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="n">
-        <v>446937</v>
+        <v>413823</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
-        <v>549989</v>
+        <v>472373</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>581390</v>
+        <v>552480</v>
       </c>
       <c r="W11" t="inlineStr"/>
     </row>
@@ -1603,43 +1603,43 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>314108373312.0554</v>
+        <v>299699841069.0864</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>250459390463.355</v>
+        <v>232929343463.4925</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>136915148.8427759</v>
+        <v>160228927.8513737</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
-        <v>9545927.863455219</v>
+        <v>8707264.924061259</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
-        <v>2621631</v>
+        <v>2249704</v>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
-        <v>564567763775.4104</v>
+        <v>532629184532.5789</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
-        <v>146461076.7062311</v>
+        <v>168936192.775435</v>
       </c>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="n">
-        <v>381673</v>
+        <v>350902</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
-        <v>473726</v>
+        <v>404410</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>500503</v>
+        <v>474461</v>
       </c>
       <c r="W12" t="inlineStr"/>
     </row>

</xml_diff>